<commit_message>
new scenario added and some methods added in filter page
</commit_message>
<xml_diff>
--- a/test-data/CourseFilter.xlsx
+++ b/test-data/CourseFilter.xlsx
@@ -80,14 +80,27 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2">
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <color auto="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color auto="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -100,43 +113,32 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
     </border>
-    <border>
-      <left>
-        <color rgb="FF000000"/>
-      </left>
-      <right>
-        <color rgb="FF000000"/>
-      </right>
-      <top>
-        <color rgb="FF000000"/>
-      </top>
-      <bottom>
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1">
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment horizontal="general" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment horizontal="general" vertical="top"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -451,7 +453,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FA37ECCB-16E9-411B-BB65-FEC9E05ABA54}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{32E44315-4A95-490F-9532-4B929BA01C6C}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <sheetData>
@@ -517,7 +519,7 @@
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>